<commit_message>
arrglando el analisis de h y m
</commit_message>
<xml_diff>
--- a/resultados/analisis_genero_tematico.xlsx
+++ b/resultados/analisis_genero_tematico.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="449">
   <si>
     <t>categoria</t>
   </si>
@@ -41,6 +41,15 @@
     <t>mayor_en</t>
   </si>
   <si>
+    <t>p_ajustado</t>
+  </si>
+  <si>
+    <t>p_ajustado_fmt</t>
+  </si>
+  <si>
+    <t>significativa_bh</t>
+  </si>
+  <si>
     <t>CALLE_IDENTIDAD</t>
   </si>
   <si>
@@ -56,12 +65,21 @@
     <t>ONOMATOPEYAS</t>
   </si>
   <si>
+    <t>0.006</t>
+  </si>
+  <si>
     <t>MOVILIDAD</t>
   </si>
   <si>
     <t>0.01</t>
   </si>
   <si>
+    <t>0.069</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
     <t>MUSICA_CULTURA</t>
   </si>
   <si>
@@ -71,6 +89,9 @@
     <t>Mujer</t>
   </si>
   <si>
+    <t>0.185</t>
+  </si>
+  <si>
     <t>DROGAS</t>
   </si>
   <si>
@@ -83,7 +104,7 @@
     <t>0.061</t>
   </si>
   <si>
-    <t>No</t>
+    <t>0.213</t>
   </si>
   <si>
     <t>RELIGION_IMAGINARIOS</t>
@@ -92,6 +113,9 @@
     <t>0.195</t>
   </si>
   <si>
+    <t>0.48</t>
+  </si>
+  <si>
     <t>DISCRIMINACION</t>
   </si>
   <si>
@@ -119,6 +143,9 @@
     <t>0.307</t>
   </si>
   <si>
+    <t>0.534</t>
+  </si>
+  <si>
     <t>SEXUALIDAD</t>
   </si>
   <si>
@@ -137,30 +164,45 @@
     <t>0.43</t>
   </si>
   <si>
+    <t>0.602</t>
+  </si>
+  <si>
     <t>GENERO_PODER</t>
   </si>
   <si>
     <t>0.527</t>
   </si>
   <si>
+    <t>0.692</t>
+  </si>
+  <si>
     <t>NOCTURNIDAD</t>
   </si>
   <si>
     <t>0.728</t>
   </si>
   <si>
+    <t>0.9</t>
+  </si>
+  <si>
     <t>EMOCIONES</t>
   </si>
   <si>
     <t>0.826</t>
   </si>
   <si>
+    <t>0.964</t>
+  </si>
+  <si>
     <t>PRESTIGIO_CONFLICTO</t>
   </si>
   <si>
     <t>0.982</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
     <t>ROMANCE</t>
   </si>
   <si>
@@ -168,9 +210,6 @@
   </si>
   <si>
     <t>VIOLENCIA</t>
-  </si>
-  <si>
-    <t>1</t>
   </si>
   <si>
     <t>año</t>
@@ -1668,10 +1707,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:11" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1696,10 +1735,19 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>2.0997</v>
@@ -1711,21 +1759,30 @@
         <v>1.1875</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F2">
         <v>0.312</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+        <v>14</v>
+      </c>
+      <c r="I2">
+        <v>5.823893908596389E-05</v>
+      </c>
+      <c r="J2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B3">
         <v>2.3623</v>
@@ -1737,21 +1794,30 @@
         <v>0.7904</v>
       </c>
       <c r="E3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F3">
         <v>0.229</v>
       </c>
       <c r="G3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
+        <v>14</v>
+      </c>
+      <c r="I3">
+        <v>0.006375773005178997</v>
+      </c>
+      <c r="J3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B4">
         <v>0.3642</v>
@@ -1763,21 +1829,30 @@
         <v>0.1706</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F4">
         <v>0.172</v>
       </c>
       <c r="G4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+        <v>14</v>
+      </c>
+      <c r="I4">
+        <v>0.06859740437064987</v>
+      </c>
+      <c r="J4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B5">
         <v>0.3693</v>
@@ -1789,21 +1864,30 @@
         <v>-0.1024</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F5">
         <v>0.138</v>
       </c>
       <c r="G5" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I5">
+        <v>0.184781012627073</v>
+      </c>
+      <c r="J5" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="B6">
         <v>0.4179</v>
@@ -1815,21 +1899,30 @@
         <v>0.209</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F6">
         <v>0.134</v>
       </c>
       <c r="G6" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+        <v>14</v>
+      </c>
+      <c r="I6">
+        <v>0.184781012627073</v>
+      </c>
+      <c r="J6" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B7">
         <v>0.4416</v>
@@ -1841,21 +1934,30 @@
         <v>0.0533</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F7">
         <v>0.125</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+        <v>14</v>
+      </c>
+      <c r="I7">
+        <v>0.2129340027669805</v>
+      </c>
+      <c r="J7" t="s">
+        <v>29</v>
+      </c>
+      <c r="K7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B8">
         <v>0.3783</v>
@@ -1867,21 +1969,30 @@
         <v>-0.2536</v>
       </c>
       <c r="E8" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F8">
         <v>0.08599999999999999</v>
       </c>
       <c r="G8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I8">
+        <v>0.4803898295699837</v>
+      </c>
+      <c r="J8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B9">
         <v>0.1512</v>
@@ -1893,21 +2004,30 @@
         <v>-0.1034</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="F9">
         <v>0.082</v>
       </c>
       <c r="G9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I9">
+        <v>0.4803898295699837</v>
+      </c>
+      <c r="J9" t="s">
+        <v>32</v>
+      </c>
+      <c r="K9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B10">
         <v>0.256</v>
@@ -1919,21 +2039,30 @@
         <v>0.055</v>
       </c>
       <c r="E10" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="F10">
         <v>0.082</v>
       </c>
       <c r="G10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+        <v>14</v>
+      </c>
+      <c r="I10">
+        <v>0.4803898295699837</v>
+      </c>
+      <c r="J10" t="s">
+        <v>32</v>
+      </c>
+      <c r="K10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B11">
         <v>0.2157</v>
@@ -1945,21 +2074,30 @@
         <v>-0.2808</v>
       </c>
       <c r="E11" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="F11">
         <v>0.08</v>
       </c>
       <c r="G11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I11">
+        <v>0.4803898295699837</v>
+      </c>
+      <c r="J11" t="s">
+        <v>32</v>
+      </c>
+      <c r="K11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="B12">
         <v>1.3235</v>
@@ -1971,21 +2109,30 @@
         <v>0.1878</v>
       </c>
       <c r="E12" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="F12">
         <v>0.076</v>
       </c>
       <c r="G12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
+        <v>14</v>
+      </c>
+      <c r="I12">
+        <v>0.4803898295699837</v>
+      </c>
+      <c r="J12" t="s">
+        <v>32</v>
+      </c>
+      <c r="K12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="B13">
         <v>0.4015</v>
@@ -1997,21 +2144,30 @@
         <v>0.1456</v>
       </c>
       <c r="E13" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F13">
         <v>0.068</v>
       </c>
       <c r="G13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
+        <v>14</v>
+      </c>
+      <c r="I13">
+        <v>0.5342871815336163</v>
+      </c>
+      <c r="J13" t="s">
+        <v>42</v>
+      </c>
+      <c r="K13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B14">
         <v>1.0252</v>
@@ -2023,21 +2179,30 @@
         <v>-0.0911</v>
       </c>
       <c r="E14" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="F14">
         <v>0.064</v>
       </c>
       <c r="G14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H14" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I14">
+        <v>0.5342871815336163</v>
+      </c>
+      <c r="J14" t="s">
+        <v>42</v>
+      </c>
+      <c r="K14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="B15">
         <v>0.9095</v>
@@ -2049,21 +2214,30 @@
         <v>-0.0673</v>
       </c>
       <c r="E15" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="F15">
         <v>0.062</v>
       </c>
       <c r="G15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I15">
+        <v>0.5342871815336163</v>
+      </c>
+      <c r="J15" t="s">
+        <v>42</v>
+      </c>
+      <c r="K15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="B16">
         <v>1.6383</v>
@@ -2075,21 +2249,30 @@
         <v>-0.1261</v>
       </c>
       <c r="E16" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="F16">
         <v>0.053</v>
       </c>
       <c r="G16" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I16">
+        <v>0.6023034823044506</v>
+      </c>
+      <c r="J16" t="s">
+        <v>49</v>
+      </c>
+      <c r="K16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B17">
         <v>2.9652</v>
@@ -2101,21 +2284,30 @@
         <v>-0.1105</v>
       </c>
       <c r="E17" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="F17">
         <v>0.042</v>
       </c>
       <c r="G17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I17">
+        <v>0.6916903843674771</v>
+      </c>
+      <c r="J17" t="s">
+        <v>52</v>
+      </c>
+      <c r="K17" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="B18">
         <v>0.5253</v>
@@ -2127,21 +2319,30 @@
         <v>0.0228</v>
       </c>
       <c r="E18" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="F18">
         <v>0.023</v>
       </c>
       <c r="G18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H18" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
+        <v>14</v>
+      </c>
+      <c r="I18">
+        <v>0.8997934900564464</v>
+      </c>
+      <c r="J18" t="s">
+        <v>55</v>
+      </c>
+      <c r="K18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="B19">
         <v>0.6486</v>
@@ -2153,21 +2354,30 @@
         <v>-0.1492</v>
       </c>
       <c r="E19" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="F19">
         <v>0.015</v>
       </c>
       <c r="G19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H19" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I19">
+        <v>0.9641950684397904</v>
+      </c>
+      <c r="J19" t="s">
+        <v>58</v>
+      </c>
+      <c r="K19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="B20">
         <v>0.214</v>
@@ -2179,21 +2389,30 @@
         <v>-0.0249</v>
       </c>
       <c r="E20" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F20">
         <v>0.002</v>
       </c>
       <c r="G20" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="J20" t="s">
+        <v>61</v>
+      </c>
+      <c r="K20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="B21">
         <v>1.3241</v>
@@ -2205,21 +2424,30 @@
         <v>-0.3805</v>
       </c>
       <c r="E21" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F21">
         <v>0.001</v>
       </c>
       <c r="G21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H21" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
+        <v>23</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="J21" t="s">
+        <v>61</v>
+      </c>
+      <c r="K21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B22">
         <v>0.1776</v>
@@ -2231,16 +2459,25 @@
         <v>-0.0106</v>
       </c>
       <c r="E22" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
       <c r="G22" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H22" t="s">
-        <v>17</v>
+        <v>23</v>
+      </c>
+      <c r="I22">
+        <v>1</v>
+      </c>
+      <c r="J22" t="s">
+        <v>61</v>
+      </c>
+      <c r="K22" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -2255,79 +2492,79 @@
   <sheetData>
     <row r="1" spans="1:25" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:25">
@@ -2335,13 +2572,13 @@
         <v>2010</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="C2" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -2412,13 +2649,13 @@
         <v>2010</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -2489,13 +2726,13 @@
         <v>2010</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -2566,13 +2803,13 @@
         <v>2010</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -2643,13 +2880,13 @@
         <v>2010</v>
       </c>
       <c r="B6" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -2720,13 +2957,13 @@
         <v>2010</v>
       </c>
       <c r="B7" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="C7" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E7">
         <v>0.6134969325153374</v>
@@ -2797,13 +3034,13 @@
         <v>2010</v>
       </c>
       <c r="B8" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -2874,13 +3111,13 @@
         <v>2010</v>
       </c>
       <c r="B9" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -2951,13 +3188,13 @@
         <v>2010</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -3028,13 +3265,13 @@
         <v>2010</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -3105,13 +3342,13 @@
         <v>2010</v>
       </c>
       <c r="B12" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="C12" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D12" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -3182,13 +3419,13 @@
         <v>2010</v>
       </c>
       <c r="B13" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="C13" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D13" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -3259,13 +3496,13 @@
         <v>2010</v>
       </c>
       <c r="B14" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C14" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D14" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -3336,13 +3573,13 @@
         <v>2010</v>
       </c>
       <c r="B15" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="C15" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -3413,13 +3650,13 @@
         <v>2010</v>
       </c>
       <c r="B16" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="C16" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D16" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -3490,13 +3727,13 @@
         <v>2011</v>
       </c>
       <c r="B17" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="D17" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -3567,13 +3804,13 @@
         <v>2011</v>
       </c>
       <c r="B18" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="C18" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D18" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -3644,13 +3881,13 @@
         <v>2011</v>
       </c>
       <c r="B19" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="D19" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -3721,13 +3958,13 @@
         <v>2011</v>
       </c>
       <c r="B20" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="C20" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="D20" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -3798,13 +4035,13 @@
         <v>2011</v>
       </c>
       <c r="B21" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="C21" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D21" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -3875,13 +4112,13 @@
         <v>2011</v>
       </c>
       <c r="B22" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="C22" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="D22" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -3952,13 +4189,13 @@
         <v>2011</v>
       </c>
       <c r="B23" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="C23" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="D23" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E23">
         <v>0.6153846153846154</v>
@@ -4029,13 +4266,13 @@
         <v>2011</v>
       </c>
       <c r="B24" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="C24" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="D24" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -4106,13 +4343,13 @@
         <v>2011</v>
       </c>
       <c r="B25" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C25" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="D25" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -4183,13 +4420,13 @@
         <v>2011</v>
       </c>
       <c r="B26" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="C26" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D26" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -4260,13 +4497,13 @@
         <v>2011</v>
       </c>
       <c r="B27" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C27" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="D27" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -4337,13 +4574,13 @@
         <v>2011</v>
       </c>
       <c r="B28" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="C28" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -4414,13 +4651,13 @@
         <v>2011</v>
       </c>
       <c r="B29" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="C29" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="D29" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -4491,13 +4728,13 @@
         <v>2011</v>
       </c>
       <c r="B30" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="C30" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="D30" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -4568,13 +4805,13 @@
         <v>2011</v>
       </c>
       <c r="B31" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="C31" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="D31" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -4645,13 +4882,13 @@
         <v>2012</v>
       </c>
       <c r="B32" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="C32" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D32" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E32">
         <v>0</v>
@@ -4722,13 +4959,13 @@
         <v>2012</v>
       </c>
       <c r="B33" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="C33" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="D33" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E33">
         <v>0</v>
@@ -4799,13 +5036,13 @@
         <v>2012</v>
       </c>
       <c r="B34" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="C34" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D34" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E34">
         <v>0</v>
@@ -4876,13 +5113,13 @@
         <v>2012</v>
       </c>
       <c r="B35" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="C35" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D35" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E35">
         <v>0</v>
@@ -4953,13 +5190,13 @@
         <v>2012</v>
       </c>
       <c r="B36" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="C36" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="D36" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -5030,13 +5267,13 @@
         <v>2012</v>
       </c>
       <c r="B37" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="C37" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="D37" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E37">
         <v>1.255230125523012</v>
@@ -5107,13 +5344,13 @@
         <v>2012</v>
       </c>
       <c r="B38" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="C38" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="D38" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E38">
         <v>0</v>
@@ -5184,13 +5421,13 @@
         <v>2012</v>
       </c>
       <c r="B39" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="C39" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="D39" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E39">
         <v>1.08695652173913</v>
@@ -5261,13 +5498,13 @@
         <v>2012</v>
       </c>
       <c r="B40" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="C40" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="D40" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E40">
         <v>0.4</v>
@@ -5338,13 +5575,13 @@
         <v>2012</v>
       </c>
       <c r="B41" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="C41" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D41" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E41">
         <v>0</v>
@@ -5415,13 +5652,13 @@
         <v>2012</v>
       </c>
       <c r="B42" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="C42" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D42" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E42">
         <v>0</v>
@@ -5492,13 +5729,13 @@
         <v>2012</v>
       </c>
       <c r="B43" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="C43" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D43" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E43">
         <v>0</v>
@@ -5569,13 +5806,13 @@
         <v>2012</v>
       </c>
       <c r="B44" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="C44" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D44" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -5646,13 +5883,13 @@
         <v>2012</v>
       </c>
       <c r="B45" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="C45" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D45" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E45">
         <v>0</v>
@@ -5723,13 +5960,13 @@
         <v>2013</v>
       </c>
       <c r="B46" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="C46" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D46" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E46">
         <v>0</v>
@@ -5800,13 +6037,13 @@
         <v>2013</v>
       </c>
       <c r="B47" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="C47" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="D47" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E47">
         <v>0</v>
@@ -5877,13 +6114,13 @@
         <v>2013</v>
       </c>
       <c r="B48" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="C48" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="D48" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -5954,13 +6191,13 @@
         <v>2013</v>
       </c>
       <c r="B49" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C49" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D49" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -6031,13 +6268,13 @@
         <v>2013</v>
       </c>
       <c r="B50" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="C50" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="D50" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E50">
         <v>0</v>
@@ -6108,13 +6345,13 @@
         <v>2013</v>
       </c>
       <c r="B51" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="C51" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D51" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E51">
         <v>0</v>
@@ -6185,13 +6422,13 @@
         <v>2013</v>
       </c>
       <c r="B52" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="C52" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="D52" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -6262,13 +6499,13 @@
         <v>2013</v>
       </c>
       <c r="B53" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="C53" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="D53" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E53">
         <v>0.7575757575757576</v>
@@ -6339,13 +6576,13 @@
         <v>2013</v>
       </c>
       <c r="B54" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="C54" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D54" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E54">
         <v>0.5602240896358543</v>
@@ -6416,13 +6653,13 @@
         <v>2013</v>
       </c>
       <c r="B55" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="C55" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="D55" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E55">
         <v>0.3048780487804878</v>
@@ -6493,13 +6730,13 @@
         <v>2013</v>
       </c>
       <c r="B56" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="C56" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D56" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -6570,13 +6807,13 @@
         <v>2013</v>
       </c>
       <c r="B57" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="C57" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D57" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -6647,13 +6884,13 @@
         <v>2013</v>
       </c>
       <c r="B58" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="C58" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="D58" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E58">
         <v>0</v>
@@ -6724,10 +6961,10 @@
         <v>2013</v>
       </c>
       <c r="C59" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="D59" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E59">
         <v>1.25</v>
@@ -6798,13 +7035,13 @@
         <v>2013</v>
       </c>
       <c r="B60" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="C60" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="D60" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -6875,13 +7112,13 @@
         <v>2014</v>
       </c>
       <c r="B61" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="C61" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D61" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -6952,13 +7189,13 @@
         <v>2014</v>
       </c>
       <c r="B62" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="C62" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D62" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E62">
         <v>0.3164556962025317</v>
@@ -7029,13 +7266,13 @@
         <v>2014</v>
       </c>
       <c r="B63" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="C63" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="D63" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E63">
         <v>1.415094339622642</v>
@@ -7106,13 +7343,13 @@
         <v>2014</v>
       </c>
       <c r="B64" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="C64" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="D64" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -7183,13 +7420,13 @@
         <v>2014</v>
       </c>
       <c r="B65" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C65" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D65" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E65">
         <v>1.183431952662722</v>
@@ -7260,13 +7497,13 @@
         <v>2014</v>
       </c>
       <c r="B66" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="C66" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="D66" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -7337,13 +7574,13 @@
         <v>2014</v>
       </c>
       <c r="B67" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="C67" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D67" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -7414,13 +7651,13 @@
         <v>2014</v>
       </c>
       <c r="B68" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="C68" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D68" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E68">
         <v>0.3194888178913738</v>
@@ -7491,13 +7728,13 @@
         <v>2014</v>
       </c>
       <c r="B69" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="C69" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D69" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E69">
         <v>0</v>
@@ -7568,13 +7805,13 @@
         <v>2014</v>
       </c>
       <c r="B70" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="C70" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="D70" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E70">
         <v>0</v>
@@ -7645,13 +7882,13 @@
         <v>2014</v>
       </c>
       <c r="B71" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="C71" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D71" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E71">
         <v>0</v>
@@ -7722,13 +7959,13 @@
         <v>2014</v>
       </c>
       <c r="B72" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="C72" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="D72" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E72">
         <v>0</v>
@@ -7799,13 +8036,13 @@
         <v>2014</v>
       </c>
       <c r="B73" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="C73" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="D73" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E73">
         <v>0</v>
@@ -7876,13 +8113,13 @@
         <v>2014</v>
       </c>
       <c r="B74" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="C74" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D74" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E74">
         <v>0</v>
@@ -7953,13 +8190,13 @@
         <v>2014</v>
       </c>
       <c r="B75" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="C75" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="D75" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E75">
         <v>0</v>
@@ -8030,13 +8267,13 @@
         <v>2015</v>
       </c>
       <c r="B76" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="C76" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D76" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E76">
         <v>0</v>
@@ -8107,13 +8344,13 @@
         <v>2015</v>
       </c>
       <c r="B77" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="C77" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D77" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E77">
         <v>2.05761316872428</v>
@@ -8184,13 +8421,13 @@
         <v>2015</v>
       </c>
       <c r="B78" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="C78" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="D78" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E78">
         <v>0</v>
@@ -8261,13 +8498,13 @@
         <v>2015</v>
       </c>
       <c r="B79" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="C79" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D79" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E79">
         <v>0</v>
@@ -8338,13 +8575,13 @@
         <v>2015</v>
       </c>
       <c r="B80" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="C80" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="D80" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E80">
         <v>0.4464285714285714</v>
@@ -8415,13 +8652,13 @@
         <v>2015</v>
       </c>
       <c r="B81" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="C81" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="D81" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E81">
         <v>0</v>
@@ -8492,13 +8729,13 @@
         <v>2015</v>
       </c>
       <c r="B82" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="C82" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="D82" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E82">
         <v>0.8547008547008548</v>
@@ -8569,13 +8806,13 @@
         <v>2015</v>
       </c>
       <c r="B83" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="C83" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="D83" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E83">
         <v>0</v>
@@ -8646,13 +8883,13 @@
         <v>2015</v>
       </c>
       <c r="B84" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="C84" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="D84" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E84">
         <v>0</v>
@@ -8723,13 +8960,13 @@
         <v>2015</v>
       </c>
       <c r="B85" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="C85" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="D85" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E85">
         <v>0</v>
@@ -8800,13 +9037,13 @@
         <v>2015</v>
       </c>
       <c r="B86" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="C86" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D86" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E86">
         <v>0</v>
@@ -8877,13 +9114,13 @@
         <v>2015</v>
       </c>
       <c r="B87" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="C87" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D87" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E87">
         <v>0</v>
@@ -8954,13 +9191,13 @@
         <v>2015</v>
       </c>
       <c r="B88" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="C88" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D88" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E88">
         <v>0</v>
@@ -9031,13 +9268,13 @@
         <v>2015</v>
       </c>
       <c r="B89" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="C89" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D89" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E89">
         <v>0</v>
@@ -9108,13 +9345,13 @@
         <v>2015</v>
       </c>
       <c r="B90" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="C90" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="D90" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E90">
         <v>1.204819277108434</v>
@@ -9185,13 +9422,13 @@
         <v>2016</v>
       </c>
       <c r="B91" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="C91" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="D91" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E91">
         <v>1.515151515151515</v>
@@ -9262,13 +9499,13 @@
         <v>2016</v>
       </c>
       <c r="B92" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="C92" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D92" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E92">
         <v>0</v>
@@ -9339,13 +9576,13 @@
         <v>2016</v>
       </c>
       <c r="B93" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="C93" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D93" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E93">
         <v>0</v>
@@ -9416,13 +9653,13 @@
         <v>2016</v>
       </c>
       <c r="B94" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="C94" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="D94" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E94">
         <v>0</v>
@@ -9493,13 +9730,13 @@
         <v>2016</v>
       </c>
       <c r="B95" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="C95" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="D95" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E95">
         <v>2.02020202020202</v>
@@ -9570,13 +9807,13 @@
         <v>2016</v>
       </c>
       <c r="B96" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="C96" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="D96" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E96">
         <v>0</v>
@@ -9647,13 +9884,13 @@
         <v>2016</v>
       </c>
       <c r="B97" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="C97" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D97" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E97">
         <v>0</v>
@@ -9724,13 +9961,13 @@
         <v>2016</v>
       </c>
       <c r="B98" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="C98" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="D98" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E98">
         <v>0</v>
@@ -9801,13 +10038,13 @@
         <v>2016</v>
       </c>
       <c r="B99" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="C99" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="D99" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E99">
         <v>0</v>
@@ -9878,13 +10115,13 @@
         <v>2016</v>
       </c>
       <c r="B100" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="C100" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D100" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E100">
         <v>0</v>
@@ -9955,13 +10192,13 @@
         <v>2016</v>
       </c>
       <c r="B101" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="C101" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D101" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E101">
         <v>0</v>
@@ -10032,13 +10269,13 @@
         <v>2016</v>
       </c>
       <c r="B102" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="C102" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="D102" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E102">
         <v>0</v>
@@ -10109,13 +10346,13 @@
         <v>2016</v>
       </c>
       <c r="B103" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="C103" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="D103" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E103">
         <v>7.82122905027933</v>
@@ -10186,13 +10423,13 @@
         <v>2016</v>
       </c>
       <c r="B104" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="C104" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="D104" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E104">
         <v>0</v>
@@ -10263,13 +10500,13 @@
         <v>2017</v>
       </c>
       <c r="B105" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="C105" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="D105" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E105">
         <v>1.470588235294118</v>
@@ -10340,13 +10577,13 @@
         <v>2017</v>
       </c>
       <c r="B106" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="C106" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D106" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E106">
         <v>0</v>
@@ -10417,13 +10654,13 @@
         <v>2017</v>
       </c>
       <c r="B107" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="C107" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="D107" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E107">
         <v>0</v>
@@ -10494,13 +10731,13 @@
         <v>2017</v>
       </c>
       <c r="B108" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
       <c r="C108" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="D108" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E108">
         <v>0</v>
@@ -10571,13 +10808,13 @@
         <v>2017</v>
       </c>
       <c r="B109" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="C109" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="D109" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E109">
         <v>0</v>
@@ -10648,13 +10885,13 @@
         <v>2017</v>
       </c>
       <c r="B110" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
       <c r="C110" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="D110" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E110">
         <v>1.851851851851852</v>
@@ -10725,13 +10962,13 @@
         <v>2017</v>
       </c>
       <c r="B111" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="C111" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
       <c r="D111" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E111">
         <v>0.6920415224913495</v>
@@ -10802,13 +11039,13 @@
         <v>2017</v>
       </c>
       <c r="B112" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="C112" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
       <c r="D112" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E112">
         <v>0</v>
@@ -10879,13 +11116,13 @@
         <v>2017</v>
       </c>
       <c r="B113" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="C113" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="D113" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E113">
         <v>0</v>
@@ -10956,13 +11193,13 @@
         <v>2017</v>
       </c>
       <c r="B114" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
       <c r="C114" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D114" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E114">
         <v>0</v>
@@ -11033,13 +11270,13 @@
         <v>2017</v>
       </c>
       <c r="B115" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="C115" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D115" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E115">
         <v>0</v>
@@ -11110,13 +11347,13 @@
         <v>2017</v>
       </c>
       <c r="B116" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="C116" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D116" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E116">
         <v>0</v>
@@ -11187,13 +11424,13 @@
         <v>2017</v>
       </c>
       <c r="B117" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
       <c r="C117" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D117" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E117">
         <v>0</v>
@@ -11264,13 +11501,13 @@
         <v>2017</v>
       </c>
       <c r="B118" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="C118" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="D118" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E118">
         <v>0</v>
@@ -11341,13 +11578,13 @@
         <v>2018</v>
       </c>
       <c r="B119" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="C119" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="D119" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E119">
         <v>0</v>
@@ -11418,13 +11655,13 @@
         <v>2018</v>
       </c>
       <c r="B120" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="C120" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="D120" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E120">
         <v>0</v>
@@ -11495,13 +11732,13 @@
         <v>2018</v>
       </c>
       <c r="B121" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
       <c r="C121" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D121" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E121">
         <v>0</v>
@@ -11572,13 +11809,13 @@
         <v>2018</v>
       </c>
       <c r="B122" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="C122" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="D122" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E122">
         <v>0</v>
@@ -11649,13 +11886,13 @@
         <v>2018</v>
       </c>
       <c r="B123" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C123" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="D123" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E123">
         <v>1.244813278008299</v>
@@ -11726,13 +11963,13 @@
         <v>2018</v>
       </c>
       <c r="B124" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="C124" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="D124" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E124">
         <v>0</v>
@@ -11803,13 +12040,13 @@
         <v>2018</v>
       </c>
       <c r="B125" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="C125" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
       <c r="D125" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E125">
         <v>1.913875598086124</v>
@@ -11880,13 +12117,13 @@
         <v>2018</v>
       </c>
       <c r="B126" t="s">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="C126" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="D126" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E126">
         <v>0</v>
@@ -11957,13 +12194,13 @@
         <v>2018</v>
       </c>
       <c r="B127" t="s">
-        <v>267</v>
+        <v>280</v>
       </c>
       <c r="C127" t="s">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="D127" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E127">
         <v>0</v>
@@ -12034,13 +12271,13 @@
         <v>2018</v>
       </c>
       <c r="B128" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
       <c r="C128" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D128" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E128">
         <v>0</v>
@@ -12111,13 +12348,13 @@
         <v>2018</v>
       </c>
       <c r="B129" t="s">
-        <v>270</v>
+        <v>283</v>
       </c>
       <c r="C129" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D129" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E129">
         <v>0</v>
@@ -12188,13 +12425,13 @@
         <v>2018</v>
       </c>
       <c r="B130" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
       <c r="C130" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="D130" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E130">
         <v>0</v>
@@ -12265,13 +12502,13 @@
         <v>2018</v>
       </c>
       <c r="B131" t="s">
-        <v>272</v>
+        <v>285</v>
       </c>
       <c r="C131" t="s">
-        <v>273</v>
+        <v>286</v>
       </c>
       <c r="D131" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E131">
         <v>0.6060606060606061</v>
@@ -12342,13 +12579,13 @@
         <v>2018</v>
       </c>
       <c r="B132" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
       <c r="C132" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="D132" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E132">
         <v>1.621621621621622</v>
@@ -12419,13 +12656,13 @@
         <v>2019</v>
       </c>
       <c r="B133" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
       <c r="C133" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="D133" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E133">
         <v>0</v>
@@ -12496,13 +12733,13 @@
         <v>2019</v>
       </c>
       <c r="B134" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="C134" t="s">
-        <v>278</v>
+        <v>291</v>
       </c>
       <c r="D134" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E134">
         <v>2.803738317757009</v>
@@ -12573,13 +12810,13 @@
         <v>2019</v>
       </c>
       <c r="B135" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
       <c r="C135" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="D135" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E135">
         <v>1.393728222996516</v>
@@ -12650,13 +12887,13 @@
         <v>2019</v>
       </c>
       <c r="B136" t="s">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="C136" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="D136" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E136">
         <v>0</v>
@@ -12727,13 +12964,13 @@
         <v>2019</v>
       </c>
       <c r="B137" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
       <c r="C137" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="D137" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E137">
         <v>0.2754820936639119</v>
@@ -12804,13 +13041,13 @@
         <v>2019</v>
       </c>
       <c r="B138" t="s">
-        <v>284</v>
+        <v>297</v>
       </c>
       <c r="C138" t="s">
-        <v>285</v>
+        <v>298</v>
       </c>
       <c r="D138" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E138">
         <v>0</v>
@@ -12881,13 +13118,13 @@
         <v>2019</v>
       </c>
       <c r="B139" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="C139" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="D139" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E139">
         <v>0</v>
@@ -12958,13 +13195,13 @@
         <v>2019</v>
       </c>
       <c r="B140" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
       <c r="C140" t="s">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="D140" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E140">
         <v>0.2590673575129534</v>
@@ -13035,13 +13272,13 @@
         <v>2019</v>
       </c>
       <c r="B141" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="C141" t="s">
-        <v>291</v>
+        <v>304</v>
       </c>
       <c r="D141" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E141">
         <v>0.5050505050505051</v>
@@ -13112,13 +13349,13 @@
         <v>2019</v>
       </c>
       <c r="B142" t="s">
-        <v>292</v>
+        <v>305</v>
       </c>
       <c r="C142" t="s">
-        <v>293</v>
+        <v>306</v>
       </c>
       <c r="D142" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E142">
         <v>0</v>
@@ -13189,13 +13426,13 @@
         <v>2019</v>
       </c>
       <c r="B143" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="C143" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="D143" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E143">
         <v>0.9345794392523363</v>
@@ -13266,13 +13503,13 @@
         <v>2019</v>
       </c>
       <c r="B144" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="C144" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="D144" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E144">
         <v>0</v>
@@ -13343,13 +13580,13 @@
         <v>2019</v>
       </c>
       <c r="B145" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
       <c r="C145" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="D145" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E145">
         <v>5.46875</v>
@@ -13420,13 +13657,13 @@
         <v>2020</v>
       </c>
       <c r="B146" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="C146" t="s">
-        <v>299</v>
+        <v>312</v>
       </c>
       <c r="D146" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E146">
         <v>1.923076923076923</v>
@@ -13497,13 +13734,13 @@
         <v>2020</v>
       </c>
       <c r="B147" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="C147" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="D147" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E147">
         <v>0.2597402597402597</v>
@@ -13574,13 +13811,13 @@
         <v>2020</v>
       </c>
       <c r="B148" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="C148" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="D148" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E148">
         <v>0</v>
@@ -13651,13 +13888,13 @@
         <v>2020</v>
       </c>
       <c r="B149" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="C149" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="D149" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E149">
         <v>1.395348837209302</v>
@@ -13728,13 +13965,13 @@
         <v>2020</v>
       </c>
       <c r="B150" t="s">
-        <v>306</v>
+        <v>319</v>
       </c>
       <c r="C150" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D150" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E150">
         <v>0.5649717514124294</v>
@@ -13805,13 +14042,13 @@
         <v>2020</v>
       </c>
       <c r="B151" t="s">
-        <v>307</v>
+        <v>320</v>
       </c>
       <c r="C151" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="D151" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E151">
         <v>2.5</v>
@@ -13882,13 +14119,13 @@
         <v>2020</v>
       </c>
       <c r="B152" t="s">
-        <v>309</v>
+        <v>322</v>
       </c>
       <c r="C152" t="s">
-        <v>310</v>
+        <v>323</v>
       </c>
       <c r="D152" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E152">
         <v>2.604166666666667</v>
@@ -13959,13 +14196,13 @@
         <v>2020</v>
       </c>
       <c r="B153" t="s">
-        <v>311</v>
+        <v>324</v>
       </c>
       <c r="C153" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
       <c r="D153" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E153">
         <v>0.2036659877800407</v>
@@ -14036,13 +14273,13 @@
         <v>2020</v>
       </c>
       <c r="B154" t="s">
-        <v>313</v>
+        <v>326</v>
       </c>
       <c r="C154" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="D154" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E154">
         <v>0</v>
@@ -14113,13 +14350,13 @@
         <v>2020</v>
       </c>
       <c r="B155" t="s">
-        <v>314</v>
+        <v>327</v>
       </c>
       <c r="C155" t="s">
-        <v>315</v>
+        <v>328</v>
       </c>
       <c r="D155" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E155">
         <v>0</v>
@@ -14190,13 +14427,13 @@
         <v>2020</v>
       </c>
       <c r="B156" t="s">
-        <v>316</v>
+        <v>329</v>
       </c>
       <c r="C156" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D156" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E156">
         <v>0.5181347150259068</v>
@@ -14267,13 +14504,13 @@
         <v>2020</v>
       </c>
       <c r="B157" t="s">
-        <v>317</v>
+        <v>330</v>
       </c>
       <c r="C157" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="D157" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E157">
         <v>0</v>
@@ -14344,13 +14581,13 @@
         <v>2020</v>
       </c>
       <c r="B158" t="s">
-        <v>318</v>
+        <v>331</v>
       </c>
       <c r="C158" t="s">
-        <v>319</v>
+        <v>332</v>
       </c>
       <c r="D158" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E158">
         <v>3.317535545023697</v>
@@ -14421,13 +14658,13 @@
         <v>2020</v>
       </c>
       <c r="B159" t="s">
-        <v>320</v>
+        <v>333</v>
       </c>
       <c r="C159" t="s">
-        <v>321</v>
+        <v>334</v>
       </c>
       <c r="D159" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E159">
         <v>0.4484304932735426</v>
@@ -14498,13 +14735,13 @@
         <v>2020</v>
       </c>
       <c r="B160" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="C160" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="D160" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E160">
         <v>0</v>
@@ -14575,13 +14812,13 @@
         <v>2021</v>
       </c>
       <c r="B161" t="s">
-        <v>324</v>
+        <v>337</v>
       </c>
       <c r="C161" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="D161" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E161">
         <v>2.923976608187134</v>
@@ -14652,13 +14889,13 @@
         <v>2021</v>
       </c>
       <c r="B162" t="s">
-        <v>326</v>
+        <v>339</v>
       </c>
       <c r="C162" t="s">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="D162" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E162">
         <v>1.31578947368421</v>
@@ -14729,13 +14966,13 @@
         <v>2021</v>
       </c>
       <c r="B163" t="s">
-        <v>328</v>
+        <v>341</v>
       </c>
       <c r="C163" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="D163" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E163">
         <v>0</v>
@@ -14806,13 +15043,13 @@
         <v>2021</v>
       </c>
       <c r="B164" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="C164" t="s">
-        <v>330</v>
+        <v>343</v>
       </c>
       <c r="D164" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E164">
         <v>0</v>
@@ -14883,13 +15120,13 @@
         <v>2021</v>
       </c>
       <c r="B165" t="s">
-        <v>331</v>
+        <v>344</v>
       </c>
       <c r="C165" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="D165" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E165">
         <v>3.225806451612903</v>
@@ -14960,13 +15197,13 @@
         <v>2021</v>
       </c>
       <c r="B166" t="s">
-        <v>332</v>
+        <v>345</v>
       </c>
       <c r="C166" t="s">
-        <v>333</v>
+        <v>346</v>
       </c>
       <c r="D166" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E166">
         <v>0</v>
@@ -15037,13 +15274,13 @@
         <v>2021</v>
       </c>
       <c r="B167" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
       <c r="C167" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
       <c r="D167" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E167">
         <v>0</v>
@@ -15114,13 +15351,13 @@
         <v>2021</v>
       </c>
       <c r="B168" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
       <c r="C168" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D168" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E168">
         <v>0</v>
@@ -15191,13 +15428,13 @@
         <v>2021</v>
       </c>
       <c r="B169" t="s">
-        <v>337</v>
+        <v>350</v>
       </c>
       <c r="C169" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D169" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E169">
         <v>0.5050505050505051</v>
@@ -15268,13 +15505,13 @@
         <v>2021</v>
       </c>
       <c r="B170" t="s">
-        <v>338</v>
+        <v>351</v>
       </c>
       <c r="C170" t="s">
-        <v>339</v>
+        <v>352</v>
       </c>
       <c r="D170" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E170">
         <v>0</v>
@@ -15345,13 +15582,13 @@
         <v>2021</v>
       </c>
       <c r="B171" t="s">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="C171" t="s">
-        <v>341</v>
+        <v>354</v>
       </c>
       <c r="D171" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E171">
         <v>0.9202453987730062</v>
@@ -15422,13 +15659,13 @@
         <v>2021</v>
       </c>
       <c r="B172" t="s">
-        <v>342</v>
+        <v>355</v>
       </c>
       <c r="C172" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="D172" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E172">
         <v>0</v>
@@ -15499,13 +15736,13 @@
         <v>2022</v>
       </c>
       <c r="B173" t="s">
-        <v>343</v>
+        <v>356</v>
       </c>
       <c r="C173" t="s">
-        <v>344</v>
+        <v>357</v>
       </c>
       <c r="D173" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E173">
         <v>0</v>
@@ -15576,13 +15813,13 @@
         <v>2022</v>
       </c>
       <c r="B174" t="s">
-        <v>345</v>
+        <v>358</v>
       </c>
       <c r="C174" t="s">
-        <v>346</v>
+        <v>359</v>
       </c>
       <c r="D174" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E174">
         <v>1.025641025641026</v>
@@ -15653,13 +15890,13 @@
         <v>2022</v>
       </c>
       <c r="B175" t="s">
-        <v>347</v>
+        <v>360</v>
       </c>
       <c r="C175" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="D175" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E175">
         <v>1.932367149758454</v>
@@ -15730,13 +15967,13 @@
         <v>2022</v>
       </c>
       <c r="B176" t="s">
-        <v>348</v>
+        <v>361</v>
       </c>
       <c r="C176" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D176" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E176">
         <v>0</v>
@@ -15807,13 +16044,13 @@
         <v>2022</v>
       </c>
       <c r="B177" t="s">
-        <v>349</v>
+        <v>362</v>
       </c>
       <c r="C177" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="D177" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E177">
         <v>0.5128205128205128</v>
@@ -15884,13 +16121,13 @@
         <v>2022</v>
       </c>
       <c r="B178" t="s">
-        <v>350</v>
+        <v>363</v>
       </c>
       <c r="C178" t="s">
-        <v>351</v>
+        <v>364</v>
       </c>
       <c r="D178" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E178">
         <v>0</v>
@@ -15961,13 +16198,13 @@
         <v>2022</v>
       </c>
       <c r="B179" t="s">
-        <v>352</v>
+        <v>365</v>
       </c>
       <c r="C179" t="s">
-        <v>353</v>
+        <v>366</v>
       </c>
       <c r="D179" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E179">
         <v>0.6644518272425249</v>
@@ -16038,13 +16275,13 @@
         <v>2022</v>
       </c>
       <c r="B180" t="s">
-        <v>354</v>
+        <v>367</v>
       </c>
       <c r="C180" t="s">
-        <v>355</v>
+        <v>368</v>
       </c>
       <c r="D180" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E180">
         <v>1.84331797235023</v>
@@ -16115,13 +16352,13 @@
         <v>2022</v>
       </c>
       <c r="B181" t="s">
-        <v>356</v>
+        <v>369</v>
       </c>
       <c r="C181" t="s">
-        <v>357</v>
+        <v>370</v>
       </c>
       <c r="D181" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E181">
         <v>3.041825095057034</v>
@@ -16192,13 +16429,13 @@
         <v>2022</v>
       </c>
       <c r="B182" t="s">
-        <v>358</v>
+        <v>371</v>
       </c>
       <c r="C182" t="s">
-        <v>359</v>
+        <v>372</v>
       </c>
       <c r="D182" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E182">
         <v>0</v>
@@ -16269,13 +16506,13 @@
         <v>2022</v>
       </c>
       <c r="B183" t="s">
-        <v>360</v>
+        <v>373</v>
       </c>
       <c r="C183" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="D183" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E183">
         <v>0.353356890459364</v>
@@ -16346,13 +16583,13 @@
         <v>2022</v>
       </c>
       <c r="B184" t="s">
-        <v>362</v>
+        <v>375</v>
       </c>
       <c r="C184" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="D184" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E184">
         <v>0</v>
@@ -16423,13 +16660,13 @@
         <v>2022</v>
       </c>
       <c r="B185" t="s">
-        <v>364</v>
+        <v>377</v>
       </c>
       <c r="C185" t="s">
-        <v>365</v>
+        <v>378</v>
       </c>
       <c r="D185" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E185">
         <v>0</v>
@@ -16500,13 +16737,13 @@
         <v>2022</v>
       </c>
       <c r="B186" t="s">
-        <v>366</v>
+        <v>379</v>
       </c>
       <c r="C186" t="s">
-        <v>367</v>
+        <v>380</v>
       </c>
       <c r="D186" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E186">
         <v>0</v>
@@ -16577,13 +16814,13 @@
         <v>2022</v>
       </c>
       <c r="B187" t="s">
-        <v>368</v>
+        <v>381</v>
       </c>
       <c r="C187" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="D187" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E187">
         <v>0.398406374501992</v>
@@ -16654,13 +16891,13 @@
         <v>2023</v>
       </c>
       <c r="B188" t="s">
-        <v>369</v>
+        <v>382</v>
       </c>
       <c r="C188" t="s">
-        <v>370</v>
+        <v>383</v>
       </c>
       <c r="D188" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E188">
         <v>0</v>
@@ -16731,13 +16968,13 @@
         <v>2023</v>
       </c>
       <c r="B189" t="s">
-        <v>371</v>
+        <v>384</v>
       </c>
       <c r="C189" t="s">
-        <v>372</v>
+        <v>385</v>
       </c>
       <c r="D189" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E189">
         <v>0</v>
@@ -16808,13 +17045,13 @@
         <v>2023</v>
       </c>
       <c r="B190" t="s">
-        <v>373</v>
+        <v>386</v>
       </c>
       <c r="C190" t="s">
-        <v>374</v>
+        <v>387</v>
       </c>
       <c r="D190" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E190">
         <v>0.6172839506172839</v>
@@ -16885,13 +17122,13 @@
         <v>2023</v>
       </c>
       <c r="B191" t="s">
-        <v>375</v>
+        <v>388</v>
       </c>
       <c r="C191" t="s">
-        <v>376</v>
+        <v>389</v>
       </c>
       <c r="D191" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E191">
         <v>0.5</v>
@@ -16962,13 +17199,13 @@
         <v>2023</v>
       </c>
       <c r="B192" t="s">
-        <v>377</v>
+        <v>390</v>
       </c>
       <c r="C192" t="s">
-        <v>378</v>
+        <v>391</v>
       </c>
       <c r="D192" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E192">
         <v>1.376146788990826</v>
@@ -17039,13 +17276,13 @@
         <v>2023</v>
       </c>
       <c r="B193" t="s">
-        <v>379</v>
+        <v>392</v>
       </c>
       <c r="C193" t="s">
-        <v>380</v>
+        <v>393</v>
       </c>
       <c r="D193" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E193">
         <v>1.463414634146342</v>
@@ -17116,13 +17353,13 @@
         <v>2023</v>
       </c>
       <c r="B194" t="s">
-        <v>381</v>
+        <v>394</v>
       </c>
       <c r="C194" t="s">
-        <v>382</v>
+        <v>395</v>
       </c>
       <c r="D194" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E194">
         <v>0.2816901408450704</v>
@@ -17193,13 +17430,13 @@
         <v>2023</v>
       </c>
       <c r="B195" t="s">
-        <v>383</v>
+        <v>396</v>
       </c>
       <c r="C195" t="s">
-        <v>384</v>
+        <v>397</v>
       </c>
       <c r="D195" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E195">
         <v>0</v>
@@ -17270,13 +17507,13 @@
         <v>2023</v>
       </c>
       <c r="B196" t="s">
-        <v>385</v>
+        <v>398</v>
       </c>
       <c r="C196" t="s">
-        <v>386</v>
+        <v>399</v>
       </c>
       <c r="D196" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E196">
         <v>0.6451612903225806</v>
@@ -17347,13 +17584,13 @@
         <v>2023</v>
       </c>
       <c r="B197" t="s">
-        <v>387</v>
+        <v>400</v>
       </c>
       <c r="C197" t="s">
-        <v>388</v>
+        <v>401</v>
       </c>
       <c r="D197" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E197">
         <v>0</v>
@@ -17424,13 +17661,13 @@
         <v>2023</v>
       </c>
       <c r="B198" t="s">
-        <v>389</v>
+        <v>402</v>
       </c>
       <c r="C198" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D198" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E198">
         <v>0.7462686567164178</v>
@@ -17501,13 +17738,13 @@
         <v>2023</v>
       </c>
       <c r="B199" t="s">
-        <v>390</v>
+        <v>403</v>
       </c>
       <c r="C199" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D199" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E199">
         <v>0</v>
@@ -17578,13 +17815,13 @@
         <v>2023</v>
       </c>
       <c r="B200" t="s">
-        <v>391</v>
+        <v>404</v>
       </c>
       <c r="C200" t="s">
-        <v>365</v>
+        <v>378</v>
       </c>
       <c r="D200" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E200">
         <v>0</v>
@@ -17655,13 +17892,13 @@
         <v>2024</v>
       </c>
       <c r="B201" t="s">
-        <v>392</v>
+        <v>405</v>
       </c>
       <c r="C201" t="s">
-        <v>393</v>
+        <v>406</v>
       </c>
       <c r="D201" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E201">
         <v>0</v>
@@ -17732,13 +17969,13 @@
         <v>2024</v>
       </c>
       <c r="B202" t="s">
-        <v>394</v>
+        <v>407</v>
       </c>
       <c r="C202" t="s">
-        <v>395</v>
+        <v>408</v>
       </c>
       <c r="D202" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E202">
         <v>0</v>
@@ -17809,13 +18046,13 @@
         <v>2024</v>
       </c>
       <c r="B203" t="s">
-        <v>396</v>
+        <v>409</v>
       </c>
       <c r="C203" t="s">
-        <v>397</v>
+        <v>410</v>
       </c>
       <c r="D203" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E203">
         <v>0</v>
@@ -17886,13 +18123,13 @@
         <v>2024</v>
       </c>
       <c r="B204" t="s">
-        <v>398</v>
+        <v>411</v>
       </c>
       <c r="C204" t="s">
-        <v>374</v>
+        <v>387</v>
       </c>
       <c r="D204" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E204">
         <v>0.5586592178770949</v>
@@ -17963,13 +18200,13 @@
         <v>2024</v>
       </c>
       <c r="B205" t="s">
-        <v>399</v>
+        <v>412</v>
       </c>
       <c r="C205" t="s">
-        <v>400</v>
+        <v>413</v>
       </c>
       <c r="D205" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E205">
         <v>2.352941176470588</v>
@@ -18040,13 +18277,13 @@
         <v>2024</v>
       </c>
       <c r="B206" t="s">
-        <v>401</v>
+        <v>414</v>
       </c>
       <c r="C206" t="s">
-        <v>402</v>
+        <v>415</v>
       </c>
       <c r="D206" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E206">
         <v>0</v>
@@ -18117,13 +18354,13 @@
         <v>2024</v>
       </c>
       <c r="B207" t="s">
-        <v>403</v>
+        <v>416</v>
       </c>
       <c r="C207" t="s">
-        <v>404</v>
+        <v>417</v>
       </c>
       <c r="D207" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E207">
         <v>0</v>
@@ -18194,13 +18431,13 @@
         <v>2024</v>
       </c>
       <c r="B208" t="s">
-        <v>405</v>
+        <v>418</v>
       </c>
       <c r="C208" t="s">
-        <v>406</v>
+        <v>419</v>
       </c>
       <c r="D208" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E208">
         <v>0</v>
@@ -18271,13 +18508,13 @@
         <v>2024</v>
       </c>
       <c r="B209" t="s">
-        <v>407</v>
+        <v>420</v>
       </c>
       <c r="C209" t="s">
-        <v>408</v>
+        <v>421</v>
       </c>
       <c r="D209" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E209">
         <v>0</v>
@@ -18348,13 +18585,13 @@
         <v>2024</v>
       </c>
       <c r="B210" t="s">
-        <v>409</v>
+        <v>422</v>
       </c>
       <c r="C210" t="s">
-        <v>410</v>
+        <v>423</v>
       </c>
       <c r="D210" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E210">
         <v>0</v>
@@ -18425,13 +18662,13 @@
         <v>2024</v>
       </c>
       <c r="B211" t="s">
-        <v>411</v>
+        <v>424</v>
       </c>
       <c r="C211" t="s">
-        <v>408</v>
+        <v>421</v>
       </c>
       <c r="D211" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E211">
         <v>1.973684210526316</v>
@@ -18502,13 +18739,13 @@
         <v>2024</v>
       </c>
       <c r="B212" t="s">
-        <v>412</v>
+        <v>425</v>
       </c>
       <c r="C212" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="D212" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E212">
         <v>0</v>
@@ -18579,13 +18816,13 @@
         <v>2024</v>
       </c>
       <c r="B213" t="s">
-        <v>414</v>
+        <v>427</v>
       </c>
       <c r="C213" t="s">
-        <v>415</v>
+        <v>428</v>
       </c>
       <c r="D213" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E213">
         <v>1.15606936416185</v>
@@ -18656,13 +18893,13 @@
         <v>2025</v>
       </c>
       <c r="B214" t="s">
-        <v>416</v>
+        <v>429</v>
       </c>
       <c r="C214" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="D214" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E214">
         <v>1.680672268907563</v>
@@ -18733,13 +18970,13 @@
         <v>2025</v>
       </c>
       <c r="B215" t="s">
-        <v>417</v>
+        <v>430</v>
       </c>
       <c r="C215" t="s">
-        <v>418</v>
+        <v>431</v>
       </c>
       <c r="D215" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E215">
         <v>1.530612244897959</v>
@@ -18810,13 +19047,13 @@
         <v>2025</v>
       </c>
       <c r="B216" t="s">
-        <v>419</v>
+        <v>432</v>
       </c>
       <c r="C216" t="s">
-        <v>420</v>
+        <v>433</v>
       </c>
       <c r="D216" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E216">
         <v>0.5128205128205128</v>
@@ -18887,13 +19124,13 @@
         <v>2025</v>
       </c>
       <c r="B217" t="s">
-        <v>421</v>
+        <v>434</v>
       </c>
       <c r="C217" t="s">
-        <v>422</v>
+        <v>435</v>
       </c>
       <c r="D217" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E217">
         <v>0</v>
@@ -18964,13 +19201,13 @@
         <v>2025</v>
       </c>
       <c r="B218" t="s">
-        <v>423</v>
+        <v>436</v>
       </c>
       <c r="C218" t="s">
-        <v>424</v>
+        <v>437</v>
       </c>
       <c r="D218" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E218">
         <v>0</v>
@@ -19041,13 +19278,13 @@
         <v>2025</v>
       </c>
       <c r="B219" t="s">
-        <v>425</v>
+        <v>438</v>
       </c>
       <c r="C219" t="s">
-        <v>426</v>
+        <v>439</v>
       </c>
       <c r="D219" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E219">
         <v>0</v>
@@ -19118,13 +19355,13 @@
         <v>2025</v>
       </c>
       <c r="B220" t="s">
-        <v>427</v>
+        <v>440</v>
       </c>
       <c r="C220" t="s">
-        <v>428</v>
+        <v>441</v>
       </c>
       <c r="D220" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E220">
         <v>0</v>
@@ -19195,13 +19432,13 @@
         <v>2025</v>
       </c>
       <c r="B221" t="s">
-        <v>429</v>
+        <v>442</v>
       </c>
       <c r="C221" t="s">
-        <v>430</v>
+        <v>443</v>
       </c>
       <c r="D221" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E221">
         <v>0</v>
@@ -19272,13 +19509,13 @@
         <v>2025</v>
       </c>
       <c r="B222" t="s">
-        <v>431</v>
+        <v>444</v>
       </c>
       <c r="C222" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D222" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E222">
         <v>0</v>
@@ -19349,13 +19586,13 @@
         <v>2025</v>
       </c>
       <c r="B223" t="s">
-        <v>432</v>
+        <v>445</v>
       </c>
       <c r="C223" t="s">
-        <v>408</v>
+        <v>421</v>
       </c>
       <c r="D223" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E223">
         <v>0</v>
@@ -19426,13 +19663,13 @@
         <v>2025</v>
       </c>
       <c r="B224" t="s">
-        <v>433</v>
+        <v>446</v>
       </c>
       <c r="C224" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D224" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E224">
         <v>0</v>
@@ -19503,13 +19740,13 @@
         <v>2025</v>
       </c>
       <c r="B225" t="s">
-        <v>434</v>
+        <v>447</v>
       </c>
       <c r="C225" t="s">
-        <v>365</v>
+        <v>378</v>
       </c>
       <c r="D225" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E225">
         <v>0</v>
@@ -19580,13 +19817,13 @@
         <v>2025</v>
       </c>
       <c r="B226" t="s">
-        <v>435</v>
+        <v>448</v>
       </c>
       <c r="C226" t="s">
-        <v>365</v>
+        <v>378</v>
       </c>
       <c r="D226" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E226">
         <v>0</v>

</xml_diff>